<commit_message>
Fixed Streamlit database path issue
</commit_message>
<xml_diff>
--- a/data/shifts.xlsx
+++ b/data/shifts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sriha\Desktop\ticket_assignment_agent\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E92AEF75-E9A6-490A-A279-151C324A126B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975A84E4-7F24-4985-AE04-85B0EA7BDEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="22">
   <si>
     <t>Assignment Group</t>
   </si>
@@ -77,17 +77,33 @@
   </si>
   <si>
     <t>Rahul</t>
+  </si>
+  <si>
+    <t>Database Support</t>
+  </si>
+  <si>
+    <t>Network Support</t>
+  </si>
+  <si>
+    <t>Vikram</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -128,13 +144,15 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -495,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0976F6-0231-4C94-8506-20F6B48FC525}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5546875" customWidth="1"/>
@@ -505,7 +523,7 @@
     <col min="5" max="5" width="6.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -522,7 +540,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -539,7 +557,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -556,7 +574,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -573,7 +591,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -590,7 +608,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -607,8 +625,73 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F7" s="3"/>
+    <row r="7" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>